<commit_message>
v1.7: apply Rounds 6-7 for tomorrow's session (slides 1-32)
New hardware slide (r22); prompts renumbered 1/7-7/7 with workbook tab renames;
S7 letter-counting currency fix (r23); S10 three-steps redesign; S11 trim; S12
Grok row; S13 abstain-vs-guess chart; S18 server-geography map (matrix removed);
S20 most-used-tools slide (r24); S22 stop-as-action; S23-25 two pairs per element;
S27/28 de-programmed toolkit; S29 split into proven-vs-myth + mirror slides (r25);
S30-S32 refinements; R14 font pass; ledger Rounds 6-7 recorded as applied.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0129XxhbHkAygGyM97mZzm9v
</commit_message>
<xml_diff>
--- a/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
+++ b/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX2-Guesses" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX3-Tokens" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX4-Handoff" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX5-Ladder" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX6-TwoSpeeds" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX7-FeatureMenu" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX8-MoE" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BONUS-Ladder" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX5-TwoSpeeds" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX6-FeatureMenu" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX7-MoE" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G2-DataAnalysis" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX-Quotes" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX-Email" sheetId="13" state="visible" r:id="rId13"/>
@@ -560,7 +560,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EX1-TwoModes .. EX8-MoE = the eight numbered course prompts · G2-DataAnalysis = the data walkthrough (uses the Data tab) · EX-Quotes = the three-quotations exercise (PDFs in the pack) · EX-Email = the inbox play (thread file in the pack) · EX-Rebuild = the Part 3 rep · PLAYBOOK = Do / Don't / Expired, with sources.</t>
+          <t>EX1-TwoModes .. EX7-MoE = the seven numbered course prompts · G2-DataAnalysis = the data walkthrough (uses the Data tab) · EX-Quotes = the three-quotations exercise (PDFs in the pack) · EX-Email = the inbox play (thread file in the pack) · EX-Rebuild = the Part 3 rep · BONUS-Ladder = a self-study triage drill · PLAYBOOK = Do / Don't / Expired, with sources.</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 8/8 · The specialist hospital, explained</t>
+          <t>Prompt 7/7 · The specialist hospital, explained</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7024,7 +7024,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 1/8 · Two modes, felt — this chat becomes your course log</t>
+          <t>Prompt 1/7 · Two modes, felt — this chat becomes your course log</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7126,7 +7126,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 2/8 · Narrowing the guesses — two separate sends</t>
+          <t>Prompt 2/7 · Narrowing the guesses — two separate sends</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7210,7 +7210,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 3/8 · Bricks, not letters</t>
+          <t>Prompt 3/7 · Bricks, not letters</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7277,7 +7277,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 4/8 · The desk — explained, then carried</t>
+          <t>Prompt 4/7 · The desk — explained, then carried</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7361,7 +7361,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 5/8 · See the rungs sort themselves</t>
+          <t>Bonus drill · The escalation ladder — see the rungs sort themselves (self-study)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7402,7 +7402,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The escalation ladder — prompt, retrieve, fine-tune — sorted live by the AI in front of you.</t>
+          <t>The escalation ladder — prompt it, feed it documents, retrain it — sorted live by the AI in front of you.</t>
         </is>
       </c>
     </row>
@@ -7445,7 +7445,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 6/8 · Same brain, two speeds</t>
+          <t>Prompt 5/7 · Same brain, two speeds</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -7563,7 +7563,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Prompt 7/8 · Ask your own product for its menu</t>
+          <t>Prompt 6/7 · Ask your own product for its menu</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>

</xml_diff>

<commit_message>
v1.10: cut most-used slide; consolidate three PDCA slides into two
Owner-directed. "What people actually use" removed (its usage stats and
standing rule condensed into the doers slide notes; r24 kept). The toolkit
loop absorbed "PDCA in practice": practice verbs in the quadrant titles,
Deming/Toyota/LEI band with portrait at the bottom; the two-layers slide
follows directly - all PDCA material now sits on two adjacent slides. The
symptom-to-element diagnosis grid moved to workbook tab EX-Rebuild with
pointers from the CHECK quadrant, the rep slide, and Part 5's run-time
grid. Part 3 divider updated (one improvement loop, not seven techniques).
Deck 71 -> 69 slides; render-verified.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0129XxhbHkAygGyM97mZzm9v
</commit_message>
<xml_diff>
--- a/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
+++ b/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
@@ -1221,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1263,49 +1263,66 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>THE REPORT</t>
+          <t>THE GRID</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Q2 returns totaled 412 units against 28,400 shipped (1.45%), up from 1.1% in Q1. Site B drove the rise; supplier packaging changes are the suspected cause. Inspection hours were flat; two corrective actions are in draft. Full breakdown by site and supplier is in the appendix table.</t>
+          <t>Inspect with this — which element failed? wrong altitude, tone, or posture -&gt; ROLE · answers a different (or vaguer) question -&gt; TASK · generically right, specifically wrong for us -&gt; CONTEXT · right content, unusable shape or length -&gt; FORMAT · doesn't match the standard in your head -&gt; EXAMPLES · confidently invented -&gt; THE OUT is missing · sprawls past what you asked -&gt; THE STOP is missing.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The 60-word fictional report both steps run on — paste it after each prompt.</t>
+          <t>The symptom-to-element diagnosis grid (moved here from the slides in v1.10) — name the failed element, fix that ONE, rerun.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>STEP 1</t>
+          <t>THE REPORT</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Summarize this report.</t>
+          <t>Q2 returns totaled 412 units against 28,400 shipped (1.45%), up from 1.1% in Q1. Site B drove the rise; supplier packaging changes are the suspected cause. Inspection hours were flat; two corrective actions are in draft. Full breakdown by site and supplier is in the appendix table.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The naive baseline — fluent, unfocused, written for nobody in particular.</t>
+          <t>The 60-word fictional report both steps run on — paste it after each prompt.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
+          <t>STEP 1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Summarize this report.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>The naive baseline — fluent, unfocused, written for nobody in particular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
           <t>STEP 2</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Your upgrade — write it yourself: add a Role, a named reader in the Task, a &lt;=80-word cap, and an Out ("if the report doesn't say, say so"). Then send it with the same report pasted.</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Same report, four elements — watch it change league. Compare with a neighbor: which ELEMENT made the difference?</t>
         </is>

</xml_diff>

<commit_message>
v1.11: redefine the Out everywhere; embed mirror art; fix pptx repair prompt
The Out's canonical definition is now three-part (condition, honest move,
surfacing) with the checkable example "anything not stated: write UNKNOWN -
never estimate; list the gaps at the end" - propagated to the anatomy slide
(formal definition in the teal band), element card, taxonomy JSON (new
default behavior option), Template Creator, taxonomy PDF, configurator
(+recalc), cheat sheet, ELEMENTS.md, field guide, workbook, and the A1/A2
template rules (UNKNOWN -> OPEN_ITEMS). Owner's mirror illustration embedded
on the flattery-bias slide at native 16:9. PowerPoint "needs repair" fixed:
negative shape extents (invalid OOXML) from two eras-slide drawings
normalized with flip transforms - file now scans clean.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0129XxhbHkAygGyM97mZzm9v
</commit_message>
<xml_diff>
--- a/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
+++ b/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Your upgrade — write it yourself: add a Role, a named reader in the Task, a &lt;=80-word cap, and an Out ("if the report doesn't say, say so"). Then send it with the same report pasted.</t>
+          <t>Your upgrade — write it yourself: add a Role, a named reader in the Task, a &lt;=80-word cap, and an Out ("anything the report doesn't state: write UNKNOWN — never estimate; list the gaps at the end"). Then send it with the same report pasted.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Give an out ("if it doesn't say, say so") + require citations</t>
+          <t>Give an out with a checkable shape ("anything not stated: write UNKNOWN — never estimate; list the gaps") + require citations</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v1.15: EX-Dashboard exercise - staged build prompts, KPI guide, vocabulary
New Course_Workbook tab EX-Dashboard (owner request): build an HTML
dashboard from the workbook's own Data tab in four staged prompts -
SHAPE (KPIs + charts + layout proposed as plain text, then stop),
BUILD (G6 pattern: single file, offline, data embedded, formulas
visible), CHECK (reconcile to the TOTAL row + hand-recompute one tile),
REFINE (one change, re-verify). Plus WHAT MAKES A KPI (decision,
formula, target, level/trend/gap) and a 20-term dashboard vocabulary,
each term with an "ask for it like this" prompt phrasing.
Pointers wired: workbook README tab list, pack header + print count,
dashboard demo slide band + speaker notes, repo README; ledger and
project state updated. Deck rebuilt, extents clean.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0129XxhbHkAygGyM97mZzm9v
</commit_message>
<xml_diff>
--- a/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
+++ b/ai-training-prompt-engineering/deliverables/exercise-data/Course_Workbook.xlsx
@@ -20,8 +20,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G2-DataAnalysis" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX-Quotes" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX-Email" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX-Report" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLAYBOOK" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX-Dashboard" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EX-Report" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLAYBOOK" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -560,7 +561,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EX1-TwoModes .. EX7-MoE = the seven numbered course prompts · G2-DataAnalysis = the data walkthrough (uses the Data tab) · EX-Quotes = the three-quotations exercise (PDFs in the pack) · EX-Email = the inbox play (thread file in the pack) · EX-Report = the Part 3 rep (your course, reported; grid + bonus rebuild drill) · BONUS-Ladder = a self-study triage drill · PLAYBOOK = Do / Don't / Expired, with sources.</t>
+          <t>EX1-TwoModes .. EX7-MoE = the seven numbered course prompts · G2-DataAnalysis = the data walkthrough (uses the Data tab) · EX-Quotes = the three-quotations exercise (PDFs in the pack) · EX-Email = the inbox play (thread file in the pack) · EX-Dashboard = the dashboard build: shape it, build it, check it (uses the Data tab; includes the dashboard vocabulary) · EX-Report = the Part 3 rep (your course, reported; grid + bonus rebuild drill) · BONUS-Ladder = a self-study triage drill · PLAYBOOK = Do / Don't / Expired, with sources.</t>
         </is>
       </c>
     </row>
@@ -1221,6 +1222,574 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="74" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Part 4 follow-on · A dashboard from data — shape it, build it, check it (uses the Data tab of THIS workbook)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>STEP</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>COPY-PASTE THIS (one cell = one prompt)</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>WHY</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>STEP 0 · SHAPE</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Work with the Data tab of this workbook (144 data rows; exclude the TOTAL row; one Inspection_Hours cell is "n/a" — treat it as missing and say so). I want a monthly supplier-quality dashboard for a plant manager who has 60 seconds. Before you build ANYTHING, propose the shape: 1) the 3-4 KPIs worth tracking — for each: a name, its exact formula from these columns, its current value, and a sensible target; 2) one chart per question the manager will actually ask — name the chart type and what is on each axis; 3) a one-line layout sketch: what sits top-left, and why. Show me the proposal and STOP — no code yet.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Design is a gate: approve KPIs and layout as PLAIN TEXT before anything renders. A wrong KPI caught here costs a sentence; caught after the dashboard circulates, it costs a retraction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>STEP 1 · BUILD</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Approved, with these changes: [your edits — or "none"]. Build it as ONE self-contained HTML file: the Data tab embedded in the file — no server, no external calls; it must open from disk, offline, on a work laptop. Views: 1) a KPI row — the tiles we agreed, each showing the value, its state vs target, and a trend arrow with the change vs the prior month; 2) the charts we agreed, filterable by Site and Supplier; 3) a sortable, searchable data table of the underlying rows. Every number computed from the embedded data — nothing hard-coded; show each KPI's formula in a tooltip or footnote so it can be audited. Anything that cannot be computed from the data: show "—", never a guess. Footer: the as-of month, the data source ("Course Workbook Data tab — fictional training data"), and an owner-and-refresh line.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>The G6 pattern. Four constraints make an AI-built tool trustworthy: single file · offline · data embedded · formulas visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>STEP 2 · CHECK</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Before I trust it: 1) reconcile — sum Units_Shipped across the data embedded in your dashboard and compare it to the TOTAL row of the Data tab; show both numbers; 2) pick one month and one site and recompute one KPI tile by hand, showing the arithmetic; 3) list every assumption the dashboard makes (the "n/a" cell, the excluded TOTAL row, any rounding). Fix any mismatch before answering.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>The trust check, same as the data walkthrough: one reconciliation anchor plus one hand-recomputed tile beats admiring the design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>STEP 3 · REFINE</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>One improvement pass: [name ONE change — e.g. "add a target line at 2% on the defect-rate trend chart" or "add last-month deltas to every tile"]. Change only that. Tell me what you changed, and re-verify any number the change touched.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Fix one element and re-run — the improvement loop, applied to software instead of prose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Needs a tool that writes and packages code — Claude (Artifacts), ChatGPT (Canvas), Gemini (Canvas), typically paid tiers; Copilot chat can't build this today. Two cautions: the file EMBEDS the data — classify and share it like the spreadsheet it came from (share the FILE, not a public link) · it is a snapshot, not a live system — for refreshing data you need a BI tool. The generic template behind this exercise is G6 in prompt-library/.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>WHAT MAKES A KPI</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>A KPI is a number someone ACTS on — not decoration. Each one needs four things:</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>A decision</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>If nobody would do anything differently when it moves, it is trivia, not a KPI — cut it.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>A formula</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Named columns, exact arithmetic — e.g. defect rate = (Defects_Found + Units_Returned) / Units_Shipped. If you can't write the formula, you can't track the number.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>A target</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>A value is a fact; value-vs-target is a status. Targets turn a dashboard from a report into an alarm.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>The trio of views</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Every KPI answers three questions: LEVEL (where are we) · TREND (which way is it moving) · GAP (how far from target). Tiles show level+gap; the chart shows trend.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>THE VOCABULARY</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Name the parts and you can ask for them — this vocabulary carries across all data-analytics and BI tools (Power BI, Tableau, Excel dashboards alike).</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>ASK FOR IT LIKE THIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Key Performance Indicator — a number tied to a decision, with a formula and a target.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>"Propose 3-4 KPIs with formula, current value and target — then stop."</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>KPI tile / stat tile</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>The big-number card in the headline row: value + vs-target state + trend arrow.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>"A KPI row of four tiles across the top."</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Hero number</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>The single most important figure, oversized — the one number a skimmer leaves with.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>"Make on-time % the hero number."</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>The change vs the previous period, shown beside the value (▲ +0.3 pt).</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>"Each tile shows the delta vs last month."</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Sparkline</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>A tiny, axis-less trend line inside a tile or table row — trend without a full chart.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>"Add a 12-month sparkline inside each tile."</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Time series</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>A line chart of a value over time — the "is it getting better?" view.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>"A monthly time series of defect rate, one line per supplier."</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Ranked bars</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>A bar chart sorted by value — the "who is biggest / worst?" view.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>"Ranked bars of return rate by site, worst first."</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Stacked bar</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>One bar split into parts — composition and total in the same mark.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>"Stack the bar by supplier so I see each site's mix."</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Heatmap</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>A grid colored by value — patterns across two dimensions at a glance (site × month).</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>"A site-by-month heatmap of on-time %."</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Target line</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>The reference line a metric should stay above or below; also called a threshold.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>"Draw the 2% target line on the trend chart."</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Traffic-light status</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Color that encodes state — on target / warning / breach — ALWAYS paired with an icon or label, never color alone.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>"Traffic-light the tiles vs target, with a label, not just color."</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Filter / slicer</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>The control that narrows every view at once (site, supplier). "Slicer" is the Power BI / Excel word.</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>"Site and Supplier filters that apply to all views."</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Date-range picker</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>The filter for time — from/to, or presets like "last 3 months".</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>"A date-range picker with a last-quarter preset."</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Cross-filtering</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Clicking a mark in one chart filters the other views to match.</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>"Clicking a site's bar should filter the trend chart."</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Drill-down</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Click a summary number to open the rows behind it.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>"Drill-down from each tile to its underlying rows."</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Tooltip</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>The detail card that appears on hover — exact values without cluttering the chart.</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>"Tooltips with exact value, n, and the formula."</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>The key mapping colors/shapes to series — every multi-series chart needs one.</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>"A legend, plus direct labels on the last points."</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Detail grid</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>The sortable, searchable table of raw rows behind the charts — the digger's view.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>"A sortable detail grid under the charts."</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>What ONE row of the data represents (here: one month × site × supplier). Every correct denominator depends on it.</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>"State the grain before proposing any KPI."</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>As-of date</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>When the data was last refreshed, stated on the page. A dashboard without one is stale-but-credible.</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>"Footer: as-of date, source, owner, refresh cadence."</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1350,7 +1919,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>